<commit_message>
Refresh BENV IZS events with lifecycle dates
</commit_message>
<xml_diff>
--- a/data/raw/benv_exports/anemia_infettiva_2026_italia.xlsx
+++ b/data/raw/benv_exports/anemia_infettiva_2026_italia.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -414,89 +414,89 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>85161</v>
+        <v>83941</v>
       </c>
       <c r="B2" t="str">
-        <v>POSITIVITA' DIAGNOSTICA</v>
+        <v>FOCOLAIO CLINICO</v>
       </c>
       <c r="C2" t="str">
-        <v>C</v>
+        <v>E</v>
       </c>
       <c r="D2" t="str">
-        <v>27/03/2026</v>
+        <v>23/03/2026</v>
       </c>
       <c r="E2" t="str">
-        <v>16/03/2026</v>
+        <v>09/03/2026</v>
       </c>
       <c r="F2" t="str">
-        <v>-</v>
+        <v>12/05/2026</v>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>CAVALLO</v>
+        <v>OVINO</v>
       </c>
       <c r="I2" t="str">
-        <v>CAPRIE</v>
+        <v>BARI SARDO</v>
       </c>
       <c r="J2" t="str">
-        <v>TO</v>
+        <v>NU</v>
       </c>
       <c r="K2" t="str">
-        <v>PIEMONTE</v>
+        <v>SARDEGNA</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>85285</v>
+        <v>82873</v>
       </c>
       <c r="B3" t="str">
-        <v>POSITIVITA' DIAGNOSTICA</v>
+        <v>FOCOLAIO CLINICO</v>
       </c>
       <c r="C3" t="str">
-        <v>C</v>
+        <v>E</v>
       </c>
       <c r="D3" t="str">
-        <v>26/06/2026</v>
+        <v>16/01/2026</v>
       </c>
       <c r="E3" t="str">
-        <v>19/06/2026</v>
+        <v>12/01/2026</v>
       </c>
       <c r="F3" t="str">
-        <v>-</v>
+        <v>27/07/2026</v>
       </c>
       <c r="G3" t="str">
         <v/>
       </c>
       <c r="H3" t="str">
-        <v>CAVALLO</v>
+        <v>OVINO</v>
       </c>
       <c r="I3" t="str">
-        <v>FISCIANO</v>
+        <v>URI</v>
       </c>
       <c r="J3" t="str">
-        <v>SA</v>
+        <v>SS</v>
       </c>
       <c r="K3" t="str">
-        <v>CAMPANIA</v>
+        <v>SARDEGNA</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>83811</v>
+        <v>85618</v>
       </c>
       <c r="B4" t="str">
-        <v>POSITIVITA' DIAGNOSTICA</v>
+        <v>FOCOLAIO CLINICO</v>
       </c>
       <c r="C4" t="str">
         <v>C</v>
       </c>
       <c r="D4" t="str">
-        <v>25/03/2026</v>
+        <v>18/06/2026</v>
       </c>
       <c r="E4" t="str">
-        <v>19/03/2026</v>
+        <v>11/06/2026</v>
       </c>
       <c r="F4" t="str">
         <v>-</v>
@@ -505,21 +505,161 @@
         <v/>
       </c>
       <c r="H4" t="str">
-        <v>CAVALLO</v>
+        <v>OVINO</v>
       </c>
       <c r="I4" t="str">
-        <v>CAPRIE</v>
+        <v>URI</v>
       </c>
       <c r="J4" t="str">
-        <v>TO</v>
+        <v>SS</v>
       </c>
       <c r="K4" t="str">
-        <v>PIEMONTE</v>
+        <v>SARDEGNA</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>83237</v>
+      </c>
+      <c r="B5" t="str">
+        <v>FOCOLAIO CLINICO</v>
+      </c>
+      <c r="C5" t="str">
+        <v>C</v>
+      </c>
+      <c r="D5" t="str">
+        <v>06/02/2026</v>
+      </c>
+      <c r="E5" t="str">
+        <v>02/02/2026</v>
+      </c>
+      <c r="F5" t="str">
+        <v>-</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>OVINO</v>
+      </c>
+      <c r="I5" t="str">
+        <v>GIAVE</v>
+      </c>
+      <c r="J5" t="str">
+        <v>SS</v>
+      </c>
+      <c r="K5" t="str">
+        <v>SARDEGNA</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>85553</v>
+      </c>
+      <c r="B6" t="str">
+        <v>FOCOLAIO CLINICO</v>
+      </c>
+      <c r="C6" t="str">
+        <v>C</v>
+      </c>
+      <c r="D6" t="str">
+        <v>20/07/2026</v>
+      </c>
+      <c r="E6" t="str">
+        <v>09/07/2026</v>
+      </c>
+      <c r="F6" t="str">
+        <v>-</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>OVINO</v>
+      </c>
+      <c r="I6" t="str">
+        <v>BARI SARDO</v>
+      </c>
+      <c r="J6" t="str">
+        <v>NU</v>
+      </c>
+      <c r="K6" t="str">
+        <v>SARDEGNA</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>85192</v>
+      </c>
+      <c r="B7" t="str">
+        <v>FOCOLAIO CLINICO</v>
+      </c>
+      <c r="C7" t="str">
+        <v>C</v>
+      </c>
+      <c r="D7" t="str">
+        <v>18/06/2026</v>
+      </c>
+      <c r="E7" t="str">
+        <v>11/06/2026</v>
+      </c>
+      <c r="F7" t="str">
+        <v>-</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>OVINO</v>
+      </c>
+      <c r="I7" t="str">
+        <v>ITTIRI</v>
+      </c>
+      <c r="J7" t="str">
+        <v>SS</v>
+      </c>
+      <c r="K7" t="str">
+        <v>SARDEGNA</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>83512</v>
+      </c>
+      <c r="B8" t="str">
+        <v>FOCOLAIO CLINICO</v>
+      </c>
+      <c r="C8" t="str">
+        <v>C</v>
+      </c>
+      <c r="D8" t="str">
+        <v>26/02/2026</v>
+      </c>
+      <c r="E8" t="str">
+        <v>22/02/2026</v>
+      </c>
+      <c r="F8" t="str">
+        <v>-</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>OVINO</v>
+      </c>
+      <c r="I8" t="str">
+        <v>GIAVE</v>
+      </c>
+      <c r="J8" t="str">
+        <v>SS</v>
+      </c>
+      <c r="K8" t="str">
+        <v>SARDEGNA</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>